<commit_message>
feat: implement asynchronous quote update feature with web scraping
- Add new API endpoint POST /api/cotacao to trigger quote updates.
- Implement quote scraping logic using cheerio for HTML parsing.
- Introduce new fields in the FundRecord schema to store quote data.
- Ensure sequential processing of valid links with error handling for failures.
- Update UI to include new columns for current value, min/max over 52 weeks.
- Implement feedback mechanisms for success, partial failures, and blocking scenarios.
- Add comprehensive tests for unit, integration, and end-to-end scenarios.
</commit_message>
<xml_diff>
--- a/fundos-para-analise.xlsx
+++ b/fundos-para-analise.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30330"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30403"/>
   <workbookPr hidePivotFieldList="1" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7a05e40ced85b24e/_Investimentos/app-analise-relatorios/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="7" documentId="8_{21696ABF-71A9-4095-905C-9B6E44F13D93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4CBE9229-90C3-49A4-BDFD-D02F5FBA4CAD}"/>
+  <xr:revisionPtr revIDLastSave="10" documentId="8_{21696ABF-71A9-4095-905C-9B6E44F13D93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{19D307CC-8354-41D6-96EA-9ADE6F341E4D}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="2505" windowWidth="21840" windowHeight="13020" xr2:uid="{120C63C4-502D-4CB6-ADAB-13736B2A05E1}"/>
   </bookViews>
@@ -741,7 +741,7 @@
         <v>48</v>
       </c>
       <c r="D3" s="3" t="str">
-        <f t="shared" ref="D3:D40" si="0">"https://statusinvest.com.br/"&amp;C3&amp;"/"&amp;LOWER(B3)</f>
+        <f>"https://statusinvest.com.br/"&amp;C3&amp;"/"&amp;LOWER(B3)</f>
         <v>https://statusinvest.com.br/etfs/qqqi11</v>
       </c>
     </row>
@@ -750,14 +750,14 @@
         <v>37</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>45</v>
+        <v>36</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>48</v>
       </c>
       <c r="D4" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>https://statusinvest.com.br/etfs/wrld11</v>
+        <f>"https://statusinvest.com.br/"&amp;C4&amp;"/"&amp;LOWER(B4)</f>
+        <v>https://statusinvest.com.br/etfs/spyi11</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
@@ -765,14 +765,14 @@
         <v>37</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>36</v>
+        <v>45</v>
       </c>
       <c r="C5" s="3" t="s">
         <v>48</v>
       </c>
       <c r="D5" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>https://statusinvest.com.br/etfs/spyi11</v>
+        <f>"https://statusinvest.com.br/"&amp;C5&amp;"/"&amp;LOWER(B5)</f>
+        <v>https://statusinvest.com.br/etfs/wrld11</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
@@ -780,14 +780,14 @@
         <v>2</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>49</v>
       </c>
       <c r="D6" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>https://statusinvest.com.br/fiagros/jgpx11</v>
+        <f>"https://statusinvest.com.br/"&amp;C6&amp;"/"&amp;LOWER(B6)</f>
+        <v>https://statusinvest.com.br/fiagros/fgaa11</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
@@ -795,14 +795,14 @@
         <v>2</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="C7" s="3" t="s">
         <v>49</v>
       </c>
       <c r="D7" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>https://statusinvest.com.br/fiagros/fgaa11</v>
+        <f>"https://statusinvest.com.br/"&amp;C7&amp;"/"&amp;LOWER(B7)</f>
+        <v>https://statusinvest.com.br/fiagros/jgpx11</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
@@ -810,14 +810,14 @@
         <v>2</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="C8" s="3" t="s">
         <v>49</v>
       </c>
       <c r="D8" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>https://statusinvest.com.br/fiagros/rura11</v>
+        <f>"https://statusinvest.com.br/"&amp;C8&amp;"/"&amp;LOWER(B8)</f>
+        <v>https://statusinvest.com.br/fiagros/knca11</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
@@ -825,14 +825,14 @@
         <v>2</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="C9" s="3" t="s">
         <v>49</v>
       </c>
       <c r="D9" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>https://statusinvest.com.br/fiagros/knca11</v>
+        <f>"https://statusinvest.com.br/"&amp;C9&amp;"/"&amp;LOWER(B9)</f>
+        <v>https://statusinvest.com.br/fiagros/rura11</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
@@ -846,7 +846,7 @@
         <v>50</v>
       </c>
       <c r="D10" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>"https://statusinvest.com.br/"&amp;C10&amp;"/"&amp;LOWER(B10)</f>
         <v>https://statusinvest.com.br/infras/bdif11</v>
       </c>
     </row>
@@ -855,14 +855,14 @@
         <v>3</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="C11" s="3" t="s">
         <v>50</v>
       </c>
       <c r="D11" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>https://statusinvest.com.br/infras/cpti11</v>
+        <f>"https://statusinvest.com.br/"&amp;C11&amp;"/"&amp;LOWER(B11)</f>
+        <v>https://statusinvest.com.br/infras/bidb11</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
@@ -870,14 +870,14 @@
         <v>3</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>17</v>
+        <v>42</v>
       </c>
       <c r="C12" s="3" t="s">
         <v>50</v>
       </c>
       <c r="D12" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>https://statusinvest.com.br/infras/bidb11</v>
+        <f>"https://statusinvest.com.br/"&amp;C12&amp;"/"&amp;LOWER(B12)</f>
+        <v>https://statusinvest.com.br/infras/cdii11</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
@@ -885,14 +885,14 @@
         <v>3</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="C13" s="3" t="s">
         <v>50</v>
       </c>
       <c r="D13" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>https://statusinvest.com.br/infras/ifra11</v>
+        <f>"https://statusinvest.com.br/"&amp;C13&amp;"/"&amp;LOWER(B13)</f>
+        <v>https://statusinvest.com.br/infras/cpti11</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
@@ -900,14 +900,14 @@
         <v>3</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>42</v>
+        <v>24</v>
       </c>
       <c r="C14" s="3" t="s">
         <v>50</v>
       </c>
       <c r="D14" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>https://statusinvest.com.br/infras/cdii11</v>
+        <f>"https://statusinvest.com.br/"&amp;C14&amp;"/"&amp;LOWER(B14)</f>
+        <v>https://statusinvest.com.br/infras/ifra11</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
@@ -921,7 +921,7 @@
         <v>50</v>
       </c>
       <c r="D15" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>"https://statusinvest.com.br/"&amp;C15&amp;"/"&amp;LOWER(B15)</f>
         <v>https://statusinvest.com.br/infras/juro11</v>
       </c>
     </row>
@@ -930,14 +930,14 @@
         <v>4</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>41</v>
+        <v>31</v>
       </c>
       <c r="C16" s="3" t="s">
         <v>51</v>
       </c>
       <c r="D16" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>https://statusinvest.com.br/fundos-imobiliarios/pcip11</v>
+        <f>"https://statusinvest.com.br/"&amp;C16&amp;"/"&amp;LOWER(B16)</f>
+        <v>https://statusinvest.com.br/fundos-imobiliarios/afhi11</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
@@ -945,14 +945,14 @@
         <v>4</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>12</v>
+        <v>46</v>
       </c>
       <c r="C17" s="3" t="s">
         <v>51</v>
       </c>
       <c r="D17" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>https://statusinvest.com.br/fundos-imobiliarios/knsc11</v>
+        <f>"https://statusinvest.com.br/"&amp;C17&amp;"/"&amp;LOWER(B17)</f>
+        <v>https://statusinvest.com.br/fundos-imobiliarios/hgcr11</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
@@ -960,14 +960,14 @@
         <v>4</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C18" s="3" t="s">
         <v>51</v>
       </c>
       <c r="D18" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>https://statusinvest.com.br/fundos-imobiliarios/afhi11</v>
+        <f>"https://statusinvest.com.br/"&amp;C18&amp;"/"&amp;LOWER(B18)</f>
+        <v>https://statusinvest.com.br/fundos-imobiliarios/kncr11</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
@@ -975,14 +975,14 @@
         <v>4</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>46</v>
+        <v>12</v>
       </c>
       <c r="C19" s="3" t="s">
         <v>51</v>
       </c>
       <c r="D19" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>https://statusinvest.com.br/fundos-imobiliarios/hgcr11</v>
+        <f>"https://statusinvest.com.br/"&amp;C19&amp;"/"&amp;LOWER(B19)</f>
+        <v>https://statusinvest.com.br/fundos-imobiliarios/knsc11</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
@@ -990,14 +990,14 @@
         <v>4</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="C20" s="3" t="s">
         <v>51</v>
       </c>
       <c r="D20" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>https://statusinvest.com.br/fundos-imobiliarios/kncr11</v>
+        <f>"https://statusinvest.com.br/"&amp;C20&amp;"/"&amp;LOWER(B20)</f>
+        <v>https://statusinvest.com.br/fundos-imobiliarios/pcip11</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
@@ -1005,14 +1005,14 @@
         <v>5</v>
       </c>
       <c r="B21" s="11" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C21" s="3" t="s">
         <v>51</v>
       </c>
       <c r="D21" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>https://statusinvest.com.br/fundos-imobiliarios/trxf11</v>
+        <f>"https://statusinvest.com.br/"&amp;C21&amp;"/"&amp;LOWER(B21)</f>
+        <v>https://statusinvest.com.br/fundos-imobiliarios/alzr11</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
@@ -1020,14 +1020,14 @@
         <v>5</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="C22" s="3" t="s">
         <v>51</v>
       </c>
       <c r="D22" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>https://statusinvest.com.br/fundos-imobiliarios/alzr11</v>
+        <f>"https://statusinvest.com.br/"&amp;C22&amp;"/"&amp;LOWER(B22)</f>
+        <v>https://statusinvest.com.br/fundos-imobiliarios/btlg11</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
@@ -1041,7 +1041,7 @@
         <v>51</v>
       </c>
       <c r="D23" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>"https://statusinvest.com.br/"&amp;C23&amp;"/"&amp;LOWER(B23)</f>
         <v>https://statusinvest.com.br/fundos-imobiliarios/hglg11</v>
       </c>
     </row>
@@ -1056,7 +1056,7 @@
         <v>51</v>
       </c>
       <c r="D24" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>"https://statusinvest.com.br/"&amp;C24&amp;"/"&amp;LOWER(B24)</f>
         <v>https://statusinvest.com.br/fundos-imobiliarios/hgru11</v>
       </c>
     </row>
@@ -1065,14 +1065,14 @@
         <v>5</v>
       </c>
       <c r="B25" s="11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C25" s="3" t="s">
         <v>51</v>
       </c>
       <c r="D25" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>https://statusinvest.com.br/fundos-imobiliarios/btlg11</v>
+        <f>"https://statusinvest.com.br/"&amp;C25&amp;"/"&amp;LOWER(B25)</f>
+        <v>https://statusinvest.com.br/fundos-imobiliarios/hsml11</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
@@ -1080,14 +1080,14 @@
         <v>5</v>
       </c>
       <c r="B26" s="11" t="s">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="C26" s="3" t="s">
         <v>51</v>
       </c>
       <c r="D26" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>https://statusinvest.com.br/fundos-imobiliarios/hsml11</v>
+        <f>"https://statusinvest.com.br/"&amp;C26&amp;"/"&amp;LOWER(B26)</f>
+        <v>https://statusinvest.com.br/fundos-imobiliarios/trxf11</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.3">
@@ -1101,7 +1101,7 @@
         <v>51</v>
       </c>
       <c r="D27" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>"https://statusinvest.com.br/"&amp;C27&amp;"/"&amp;LOWER(B27)</f>
         <v>https://statusinvest.com.br/fundos-imobiliarios/xpml11</v>
       </c>
     </row>
@@ -1110,14 +1110,14 @@
         <v>43</v>
       </c>
       <c r="B28" s="13" t="s">
-        <v>6</v>
+        <v>38</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="D28" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>https://statusinvest.com.br/fundos-imobiliarios/urpr11</v>
+        <f>"https://statusinvest.com.br/"&amp;C28&amp;"/"&amp;LOWER(B28)</f>
+        <v>https://statusinvest.com.br/etfs/alug11</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.3">
@@ -1128,11 +1128,11 @@
         <v>11</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D29" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>https://statusinvest.com.br/fundos-imobiliarios/gcra11</v>
+        <f>"https://statusinvest.com.br/"&amp;C29&amp;"/"&amp;LOWER(B29)</f>
+        <v>https://statusinvest.com.br/fiagros/gcra11</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.3">
@@ -1140,14 +1140,14 @@
         <v>43</v>
       </c>
       <c r="B30" s="13" t="s">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="C30" s="3" t="s">
         <v>51</v>
       </c>
       <c r="D30" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>https://statusinvest.com.br/fundos-imobiliarios/ibcr11</v>
+        <f>"https://statusinvest.com.br/"&amp;C30&amp;"/"&amp;LOWER(B30)</f>
+        <v>https://statusinvest.com.br/fundos-imobiliarios/brcr11</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.3">
@@ -1155,14 +1155,14 @@
         <v>43</v>
       </c>
       <c r="B31" s="13" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="C31" s="3" t="s">
         <v>51</v>
       </c>
       <c r="D31" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>https://statusinvest.com.br/fundos-imobiliarios/rbrp11</v>
+        <f>"https://statusinvest.com.br/"&amp;C31&amp;"/"&amp;LOWER(B31)</f>
+        <v>https://statusinvest.com.br/fundos-imobiliarios/btra11</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.3">
@@ -1170,14 +1170,14 @@
         <v>43</v>
       </c>
       <c r="B32" s="13" t="s">
-        <v>27</v>
+        <v>39</v>
       </c>
       <c r="C32" s="3" t="s">
         <v>51</v>
       </c>
       <c r="D32" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>https://statusinvest.com.br/fundos-imobiliarios/brcr11</v>
+        <f>"https://statusinvest.com.br/"&amp;C32&amp;"/"&amp;LOWER(B32)</f>
+        <v>https://statusinvest.com.br/fundos-imobiliarios/fyto11</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.3">
@@ -1185,14 +1185,14 @@
         <v>43</v>
       </c>
       <c r="B33" s="13" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C33" s="3" t="s">
         <v>51</v>
       </c>
       <c r="D33" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>https://statusinvest.com.br/fundos-imobiliarios/btra11</v>
+        <f>"https://statusinvest.com.br/"&amp;C33&amp;"/"&amp;LOWER(B33)</f>
+        <v>https://statusinvest.com.br/fundos-imobiliarios/gcri11</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.3">
@@ -1200,29 +1200,29 @@
         <v>43</v>
       </c>
       <c r="B34" s="13" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="C34" s="3" t="s">
         <v>51</v>
       </c>
       <c r="D34" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>https://statusinvest.com.br/fundos-imobiliarios/fyto11</v>
+        <f>"https://statusinvest.com.br/"&amp;C34&amp;"/"&amp;LOWER(B34)</f>
+        <v>https://statusinvest.com.br/fundos-imobiliarios/hgre11</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A35" s="8" t="s">
+      <c r="A35" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="B35" s="9" t="s">
-        <v>8</v>
+      <c r="B35" s="13" t="s">
+        <v>9</v>
       </c>
       <c r="C35" s="3" t="s">
         <v>51</v>
       </c>
       <c r="D35" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>https://statusinvest.com.br/fundos-imobiliarios/rbrr11</v>
+        <f>"https://statusinvest.com.br/"&amp;C35&amp;"/"&amp;LOWER(B35)</f>
+        <v>https://statusinvest.com.br/fundos-imobiliarios/ibcr11</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.3">
@@ -1230,14 +1230,14 @@
         <v>43</v>
       </c>
       <c r="B36" s="13" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C36" s="3" t="s">
         <v>51</v>
       </c>
       <c r="D36" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>https://statusinvest.com.br/fundos-imobiliarios/gcri11</v>
+        <f>"https://statusinvest.com.br/"&amp;C36&amp;"/"&amp;LOWER(B36)</f>
+        <v>https://statusinvest.com.br/fundos-imobiliarios/rbrl11</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.3">
@@ -1245,29 +1245,29 @@
         <v>43</v>
       </c>
       <c r="B37" s="13" t="s">
-        <v>38</v>
+        <v>29</v>
       </c>
       <c r="C37" s="3" t="s">
         <v>51</v>
       </c>
       <c r="D37" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>https://statusinvest.com.br/fundos-imobiliarios/alug11</v>
+        <f>"https://statusinvest.com.br/"&amp;C37&amp;"/"&amp;LOWER(B37)</f>
+        <v>https://statusinvest.com.br/fundos-imobiliarios/rbrp11</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A38" s="12" t="s">
+      <c r="A38" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="B38" s="13" t="s">
-        <v>22</v>
+      <c r="B38" s="9" t="s">
+        <v>8</v>
       </c>
       <c r="C38" s="3" t="s">
         <v>51</v>
       </c>
       <c r="D38" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>https://statusinvest.com.br/fundos-imobiliarios/rbrl11</v>
+        <f>"https://statusinvest.com.br/"&amp;C38&amp;"/"&amp;LOWER(B38)</f>
+        <v>https://statusinvest.com.br/fundos-imobiliarios/rbrr11</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.3">
@@ -1275,14 +1275,14 @@
         <v>43</v>
       </c>
       <c r="B39" s="13" t="s">
-        <v>34</v>
+        <v>6</v>
       </c>
       <c r="C39" s="3" t="s">
         <v>51</v>
       </c>
       <c r="D39" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>https://statusinvest.com.br/fundos-imobiliarios/hgre11</v>
+        <f>"https://statusinvest.com.br/"&amp;C39&amp;"/"&amp;LOWER(B39)</f>
+        <v>https://statusinvest.com.br/fundos-imobiliarios/urpr11</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.3">
@@ -1296,11 +1296,16 @@
         <v>50</v>
       </c>
       <c r="D40" s="3" t="str">
-        <f t="shared" si="0"/>
+        <f>"https://statusinvest.com.br/"&amp;C40&amp;"/"&amp;LOWER(B40)</f>
         <v>https://statusinvest.com.br/infras/bodb11</v>
       </c>
     </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D40">
+    <sortCondition ref="A2:A40"/>
+    <sortCondition ref="C2:C40"/>
+    <sortCondition ref="B2:B40"/>
+  </sortState>
   <conditionalFormatting sqref="A2:A33">
     <cfRule type="cellIs" dxfId="1" priority="1" operator="lessThan">
       <formula>0</formula>

</xml_diff>